<commit_message>
fix(preprocessing): Quitar comillas innecesarias en campos de texto
</commit_message>
<xml_diff>
--- a/data/processed/BAI_PROCESSED.xlsx
+++ b/data/processed/BAI_PROCESSED.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -655,7 +655,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -746,7 +746,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -837,7 +837,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -928,7 +928,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4396,7 +4396,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F60" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -6024,7 +6024,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -6216,7 +6216,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -6398,7 +6398,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -6479,7 +6479,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -6489,7 +6489,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -6580,7 +6580,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -6661,7 +6661,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6671,7 +6671,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -6944,7 +6944,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -7025,7 +7025,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -7116,7 +7116,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7126,7 +7126,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -7207,7 +7207,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -7389,7 +7389,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -7480,7 +7480,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7672,7 +7672,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -7763,7 +7763,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7945,7 +7945,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -8036,7 +8036,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -8218,7 +8218,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -8309,7 +8309,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -8491,7 +8491,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -8572,7 +8572,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>"severe"</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8855,7 +8855,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -9037,7 +9037,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -9118,7 +9118,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -9128,7 +9128,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -9209,7 +9209,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -9310,7 +9310,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -9391,7 +9391,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -9401,7 +9401,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -9492,7 +9492,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -9573,7 +9573,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -9583,7 +9583,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -9765,7 +9765,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -9856,7 +9856,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -9937,7 +9937,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -9947,7 +9947,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F105" t="n">
@@ -10028,7 +10028,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -10129,7 +10129,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -10210,7 +10210,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F108" t="n">
@@ -10301,7 +10301,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -10392,7 +10392,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F110" t="n">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>"moderate"</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -10493,7 +10493,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -10574,7 +10574,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -10584,7 +10584,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F112" t="n">
@@ -10665,7 +10665,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -10675,7 +10675,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -10756,7 +10756,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -10766,7 +10766,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>"F"</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>"low"</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -10857,7 +10857,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>"M"</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F115" t="n">

</xml_diff>